<commit_message>
Rechnung Fahrrad: USt-IdNr. entfernt, nur Steuernummer
Die Fusszeile nennt jetzt allein die Steuernummer 26 026 70812, Finanzamt
Mainz-Sued. Nach Paragraf 14 UStG genuegt das; eine USt-IdNr. ist keine
zusaetzliche Pflichtangabe. Der Hinweis zur fremden USt-IdNr. entfaellt
damit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-rechnung-fahrrad-sascha-an-holding.xlsx
+++ b/10_Output/2026-10-21-rechnung-fahrrad-sascha-an-holding.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Rechnung" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Rechnung!$A$1:$I$36</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Rechnung!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
   <si>
     <t xml:space="preserve">Sascha Coldewey</t>
   </si>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Sascha Coldewey · Im Zuckergarten 28 · 55129 Mainz</t>
   </si>
   <si>
-    <t xml:space="preserve">Steuernummer 26 026 70812 · Finanzamt Mainz-Süd · USt-IdNr. DE278832927</t>
+    <t xml:space="preserve">Steuernummer 26 026 70812 · Finanzamt Mainz-Süd</t>
   </si>
   <si>
     <t xml:space="preserve">Vor dem Versenden prüfen</t>
@@ -163,31 +163,25 @@
     <t xml:space="preserve">OFFEN</t>
   </si>
   <si>
-    <t xml:space="preserve">USt-IdNr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE278832927 ist auf der Flugrechnung vom August als USt-IdNr. der Coldewey Holding GmbH ausgewiesen. Auf einer Rechnung von dir an die Holding muss deine eigene Nummer stehen, sonst wären Aussteller und Empfänger derselbe Unternehmer. Hast du keine eigene, lass die Zeile weg — die Steuernummer allein genügt als Pflichtangabe.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Verkauf an die eigene GmbH</t>
   </si>
   <si>
     <t xml:space="preserve">Der Preis muss dem entsprechen, was ein Fremder zahlen würde. Ein fünf Monate altes Rad zum vollen Neupreis kann das Finanzamt als verdeckte Gewinnausschüttung werten. Üblich ist ein Abschlag; den Preis im Zweifel über Vergleichsangebote belegen und die Rose-Rechnung beilegen.</t>
   </si>
   <si>
-    <t xml:space="preserve">Trittst du als Unternehmer auf?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mit ausgewiesener Umsatzsteuer ist das ein unternehmerischer Verkauf, kein privater. Verkaufst du wirklich aus dem Privatvermögen, darf keine Umsatzsteuer auf der Rechnung stehen — die Holding kann dann aber auch keine Vorsteuer ziehen. Beides zusammen geht nicht.</t>
-  </si>
-  <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
+    <t xml:space="preserve">Unternehmerischer Verkauf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mit Steuernummer und ausgewiesener Umsatzsteuer rechnest du als Unternehmer ab, nicht aus dem Privatvermögen. Die Holding kann die 391,01 € als Vorsteuer ziehen, und du meldest sie in deiner Umsatzsteuervoranmeldung an.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pflichtangaben</t>
   </si>
   <si>
-    <t xml:space="preserve">Nach § 14 UStG fehlen noch Rechnungsnummer und Leistungsdatum, beide oben gelb. Alles Übrige ist enthalten: Namen und Anschriften, Steuernummer, Menge und Art, Entgelt, Steuersatz und Steuerbetrag.</t>
+    <t xml:space="preserve">Nach § 14 UStG fehlen noch Rechnungsnummer und Leistungsdatum, beide oben gelb. Alles Übrige ist enthalten: Namen und Anschriften, Steuernummer, Menge und Art, Entgelt, Steuersatz und Steuerbetrag. Die Steuernummer genügt, eine USt-IdNr. ist ausdrücklich keine zusätzliche Pflicht.</t>
   </si>
 </sst>
 </file>
@@ -781,7 +775,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1054,58 +1048,41 @@
       <c r="I32" s="26"/>
     </row>
     <row r="33" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" s="25" t="s">
+      <c r="A33" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="B33" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
+      <c r="C33" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
     </row>
     <row r="34" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="B34" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" s="26" t="s">
+      <c r="A34" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-    </row>
-    <row r="35" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="27" t="s">
+      <c r="C34" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="C35" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
-      <c r="G35" s="29"/>
-      <c r="H35" s="29"/>
-      <c r="I35" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="15">
     <mergeCell ref="G1:I2"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="G7:I7"/>
@@ -1121,7 +1098,6 @@
     <mergeCell ref="C32:I32"/>
     <mergeCell ref="C33:I33"/>
     <mergeCell ref="C34:I34"/>
-    <mergeCell ref="C35:I35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>